<commit_message>
Enemy moves, new issue put on excel
Enemy can now move itself to the first location. Made a mistake when typing a line of code, documented on excel now.
</commit_message>
<xml_diff>
--- a/Assets/TestPlanTemplate.xlsx
+++ b/Assets/TestPlanTemplate.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\ZakUnityFMP\FMP Concepts\Assets\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\UnityZakFMP\FMP-Concepts\Assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{51005DF5-10C4-4CC9-A627-CC5C6003E09C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E7BA0BC9-2CE3-474C-9F7B-37123D2536D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="209" xr2:uid="{D9B1ECAE-43F8-4EE8-A9A6-870A8BC1A0C0}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="108" xr2:uid="{D9B1ECAE-43F8-4EE8-A9A6-870A8BC1A0C0}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="33">
   <si>
     <t>Test Number</t>
   </si>
@@ -145,14 +145,26 @@
     <t>Required System.Collections.Generic; which wasn't previously there</t>
   </si>
   <si>
-    <t>Assets\Scripts\BasicAiEnemyBehaviour\EnemyBehaviour.cs(8,12): error CS0246: The type or namespace name 'List&lt;&gt;' could not be found (are you missing a using directive or an assembly reference?)</t>
+    <t>Moving the Enemy</t>
+  </si>
+  <si>
+    <t>Enemy moves to first patrol point</t>
+  </si>
+  <si>
+    <t>Assets\Scripts\BasicAiEnemyBehaviour\EnemyBehaviour.cs(17,9): error CS0103: The name 'MoveToNextPatrolRoute' does not exist in the current context</t>
+  </si>
+  <si>
+    <t>The type or namespace name 'List&lt;&gt;' could not be found (are you missing a using directive or an assembly reference?)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Typed "MoveToNextPatrolRoute();" when I was meant to </t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="18"/>
       <color theme="1"/>
@@ -180,6 +192,12 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="18"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="4">
@@ -229,7 +247,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -243,20 +261,17 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -593,7 +608,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{578B1A4F-6B1D-4B59-8AFF-2D563D27525C}">
   <dimension ref="A1:H101"/>
-  <sheetFormatPr defaultRowHeight="24" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="23.25" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="8.6640625" style="3"/>
     <col min="2" max="2" width="15.6640625" style="4" customWidth="1"/>
@@ -606,14 +621,14 @@
     <col min="9" max="16384" width="8.6640625" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="36" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:8" ht="36" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="6" t="s">
+      <c r="B1" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="C1" s="5" t="s">
+      <c r="C1" s="8" t="s">
         <v>8</v>
       </c>
       <c r="D1" s="1" t="s">
@@ -632,11 +647,11 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A2" s="3">
         <v>1</v>
       </c>
-      <c r="B2" s="7" t="s">
+      <c r="B2" s="6" t="s">
         <v>6</v>
       </c>
       <c r="C2" s="4" t="s">
@@ -656,7 +671,7 @@
       </c>
       <c r="H2" s="4"/>
     </row>
-    <row r="3" spans="1:8" ht="48" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:8" ht="46.5" x14ac:dyDescent="0.35">
       <c r="A3" s="3">
         <v>2</v>
       </c>
@@ -682,7 +697,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="48" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:8" ht="46.5" x14ac:dyDescent="0.35">
       <c r="A4" s="3">
         <v>3</v>
       </c>
@@ -692,7 +707,7 @@
       <c r="C4" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="D4" s="8" t="s">
+      <c r="D4" s="4" t="s">
         <v>7</v>
       </c>
       <c r="F4" s="4" t="s">
@@ -705,7 +720,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A5" s="3">
         <v>4</v>
       </c>
@@ -728,7 +743,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="72" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:8" ht="46.5" x14ac:dyDescent="0.35">
       <c r="A6" s="3">
         <v>5</v>
       </c>
@@ -742,577 +757,594 @@
         <v>22</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="H6" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="H6" s="7" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:8" ht="46.5" x14ac:dyDescent="0.35">
       <c r="A7" s="3">
         <v>6</v>
       </c>
-      <c r="F7" s="4"/>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="B7" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="F7" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="G7" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="H7" s="2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A8" s="3">
         <v>7</v>
       </c>
       <c r="F8" s="4"/>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A9" s="3">
         <v>8</v>
       </c>
       <c r="F9" s="4"/>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A10" s="3">
         <v>9</v>
       </c>
       <c r="F10" s="4"/>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A11" s="3">
         <v>10</v>
       </c>
       <c r="F11" s="4"/>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A12" s="3">
         <v>11</v>
       </c>
       <c r="F12" s="4"/>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A13" s="3">
         <v>12</v>
       </c>
       <c r="F13" s="4"/>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A14" s="3">
         <v>13</v>
       </c>
       <c r="F14" s="4"/>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A15" s="3">
         <v>14</v>
       </c>
       <c r="F15" s="4"/>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A16" s="3">
         <v>15</v>
       </c>
       <c r="F16" s="4"/>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A17" s="3">
         <v>16</v>
       </c>
       <c r="F17" s="4"/>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A18" s="3">
         <v>17</v>
       </c>
       <c r="F18" s="4"/>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A19" s="3">
         <v>18</v>
       </c>
       <c r="F19" s="4"/>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A20" s="3">
         <v>19</v>
       </c>
       <c r="F20" s="4"/>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A21" s="3">
         <v>20</v>
       </c>
       <c r="F21" s="4"/>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A22" s="3">
         <v>21</v>
       </c>
       <c r="F22" s="4"/>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A23" s="3">
         <v>22</v>
       </c>
       <c r="F23" s="4"/>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A24" s="3">
         <v>23</v>
       </c>
       <c r="F24" s="4"/>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A25" s="3">
         <v>24</v>
       </c>
       <c r="F25" s="4"/>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A26" s="3">
         <v>25</v>
       </c>
       <c r="F26" s="4"/>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A27" s="3">
         <v>26</v>
       </c>
       <c r="F27" s="4"/>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A28" s="3">
         <v>27</v>
       </c>
       <c r="F28" s="4"/>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A29" s="3">
         <v>28</v>
       </c>
       <c r="F29" s="4"/>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A30" s="3">
         <v>29</v>
       </c>
       <c r="F30" s="4"/>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A31" s="3">
         <v>30</v>
       </c>
       <c r="F31" s="4"/>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A32" s="3">
         <v>31</v>
       </c>
       <c r="F32" s="4"/>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A33" s="3">
         <v>32</v>
       </c>
       <c r="F33" s="4"/>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="34" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A34" s="3">
         <v>33</v>
       </c>
       <c r="F34" s="4"/>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="35" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A35" s="3">
         <v>34</v>
       </c>
       <c r="F35" s="4"/>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="36" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A36" s="3">
         <v>35</v>
       </c>
       <c r="F36" s="4"/>
     </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="37" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A37" s="3">
         <v>36</v>
       </c>
       <c r="F37" s="4"/>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="38" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A38" s="3">
         <v>37</v>
       </c>
       <c r="F38" s="4"/>
     </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="39" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A39" s="3">
         <v>38</v>
       </c>
       <c r="F39" s="4"/>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="40" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A40" s="3">
         <v>39</v>
       </c>
       <c r="F40" s="4"/>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="41" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A41" s="3">
         <v>40</v>
       </c>
       <c r="F41" s="4"/>
     </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="42" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A42" s="3">
         <v>41</v>
       </c>
       <c r="F42" s="4"/>
     </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="43" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A43" s="3">
         <v>42</v>
       </c>
       <c r="F43" s="4"/>
     </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="44" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A44" s="3">
         <v>43</v>
       </c>
       <c r="F44" s="4"/>
     </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="45" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A45" s="3">
         <v>44</v>
       </c>
       <c r="F45" s="4"/>
     </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="46" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A46" s="3">
         <v>45</v>
       </c>
       <c r="F46" s="4"/>
     </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="47" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A47" s="3">
         <v>46</v>
       </c>
       <c r="F47" s="4"/>
     </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="48" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A48" s="3">
         <v>47</v>
       </c>
       <c r="F48" s="4"/>
     </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="49" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A49" s="3">
         <v>48</v>
       </c>
       <c r="F49" s="4"/>
     </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="50" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A50" s="3">
         <v>49</v>
       </c>
       <c r="F50" s="4"/>
     </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="51" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A51" s="3">
         <v>50</v>
       </c>
       <c r="F51" s="4"/>
     </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="52" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A52" s="3">
         <v>51</v>
       </c>
       <c r="F52" s="4"/>
     </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="53" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A53" s="3">
         <v>52</v>
       </c>
       <c r="F53" s="4"/>
     </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="54" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A54" s="3">
         <v>53</v>
       </c>
       <c r="F54" s="4"/>
     </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="55" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A55" s="3">
         <v>54</v>
       </c>
       <c r="F55" s="4"/>
     </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="56" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A56" s="3">
         <v>55</v>
       </c>
       <c r="F56" s="4"/>
     </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="57" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A57" s="3">
         <v>56</v>
       </c>
       <c r="F57" s="4"/>
     </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="58" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A58" s="3">
         <v>57</v>
       </c>
       <c r="F58" s="4"/>
     </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="59" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A59" s="3">
         <v>58</v>
       </c>
       <c r="F59" s="4"/>
     </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="60" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A60" s="3">
         <v>59</v>
       </c>
       <c r="F60" s="4"/>
     </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="61" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A61" s="3">
         <v>60</v>
       </c>
       <c r="F61" s="4"/>
     </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="62" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A62" s="3">
         <v>61</v>
       </c>
       <c r="F62" s="4"/>
     </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="63" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A63" s="3">
         <v>62</v>
       </c>
       <c r="F63" s="4"/>
     </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="64" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A64" s="3">
         <v>63</v>
       </c>
       <c r="F64" s="4"/>
     </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="65" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A65" s="3">
         <v>64</v>
       </c>
       <c r="F65" s="4"/>
     </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="66" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A66" s="3">
         <v>65</v>
       </c>
       <c r="F66" s="4"/>
     </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="67" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A67" s="3">
         <v>66</v>
       </c>
       <c r="F67" s="4"/>
     </row>
-    <row r="68" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="68" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A68" s="3">
         <v>67</v>
       </c>
       <c r="F68" s="4"/>
     </row>
-    <row r="69" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="69" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A69" s="3">
         <v>68</v>
       </c>
       <c r="F69" s="4"/>
     </row>
-    <row r="70" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="70" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A70" s="3">
         <v>69</v>
       </c>
       <c r="F70" s="4"/>
     </row>
-    <row r="71" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="71" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A71" s="3">
         <v>70</v>
       </c>
       <c r="F71" s="4"/>
     </row>
-    <row r="72" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="72" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A72" s="3">
         <v>71</v>
       </c>
       <c r="F72" s="4"/>
     </row>
-    <row r="73" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="73" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A73" s="3">
         <v>72</v>
       </c>
       <c r="F73" s="4"/>
     </row>
-    <row r="74" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="74" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A74" s="3">
         <v>73</v>
       </c>
       <c r="F74" s="4"/>
     </row>
-    <row r="75" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="75" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A75" s="3">
         <v>74</v>
       </c>
       <c r="F75" s="4"/>
     </row>
-    <row r="76" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="76" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A76" s="3">
         <v>75</v>
       </c>
       <c r="F76" s="4"/>
     </row>
-    <row r="77" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="77" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A77" s="3">
         <v>76</v>
       </c>
       <c r="F77" s="4"/>
     </row>
-    <row r="78" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="78" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A78" s="3">
         <v>77</v>
       </c>
       <c r="F78" s="4"/>
     </row>
-    <row r="79" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="79" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A79" s="3">
         <v>78</v>
       </c>
       <c r="F79" s="4"/>
     </row>
-    <row r="80" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="80" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A80" s="3">
         <v>79</v>
       </c>
       <c r="F80" s="4"/>
     </row>
-    <row r="81" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="81" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A81" s="3">
         <v>80</v>
       </c>
       <c r="F81" s="4"/>
     </row>
-    <row r="82" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="82" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A82" s="3">
         <v>81</v>
       </c>
       <c r="F82" s="4"/>
     </row>
-    <row r="83" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="83" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A83" s="3">
         <v>82</v>
       </c>
       <c r="F83" s="4"/>
     </row>
-    <row r="84" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="84" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A84" s="3">
         <v>83</v>
       </c>
       <c r="F84" s="4"/>
     </row>
-    <row r="85" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="85" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A85" s="3">
         <v>84</v>
       </c>
       <c r="F85" s="4"/>
     </row>
-    <row r="86" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="86" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A86" s="3">
         <v>85</v>
       </c>
       <c r="F86" s="4"/>
     </row>
-    <row r="87" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="87" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A87" s="3">
         <v>86</v>
       </c>
       <c r="F87" s="4"/>
     </row>
-    <row r="88" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="88" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A88" s="3">
         <v>87</v>
       </c>
       <c r="F88" s="4"/>
     </row>
-    <row r="89" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="89" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A89" s="3">
         <v>88</v>
       </c>
       <c r="F89" s="4"/>
     </row>
-    <row r="90" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="90" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A90" s="3">
         <v>89</v>
       </c>
       <c r="F90" s="4"/>
     </row>
-    <row r="91" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="91" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A91" s="3">
         <v>90</v>
       </c>
       <c r="F91" s="4"/>
     </row>
-    <row r="92" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="92" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A92" s="3">
         <v>91</v>
       </c>
       <c r="F92" s="4"/>
     </row>
-    <row r="93" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="93" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A93" s="3">
         <v>92</v>
       </c>
       <c r="F93" s="4"/>
     </row>
-    <row r="94" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="94" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A94" s="3">
         <v>93</v>
       </c>
       <c r="F94" s="4"/>
     </row>
-    <row r="95" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="95" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A95" s="3">
         <v>94</v>
       </c>
       <c r="F95" s="4"/>
     </row>
-    <row r="96" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="96" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A96" s="3">
         <v>95</v>
       </c>
       <c r="F96" s="4"/>
     </row>
-    <row r="97" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="97" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A97" s="3">
         <v>96</v>
       </c>
       <c r="F97" s="4"/>
     </row>
-    <row r="98" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="98" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A98" s="3">
         <v>97</v>
       </c>
       <c r="F98" s="4"/>
     </row>
-    <row r="99" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="99" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A99" s="3">
         <v>98</v>
       </c>
       <c r="F99" s="4"/>
     </row>
-    <row r="100" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="100" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A100" s="3">
         <v>99</v>
       </c>
       <c r="F100" s="4"/>
     </row>
-    <row r="101" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="101" spans="1:6" x14ac:dyDescent="0.35">
       <c r="F101" s="4"/>
     </row>
   </sheetData>
@@ -1322,26 +1354,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="f2c92a4b-fdf1-4091-a3b5-730e0262f810">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="ed40aa6c-982d-4d5a-abf0-52239ff24e20" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100CBBF1B2C966E054EA174FC74AC82655E" ma:contentTypeVersion="11" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="8c104540bbb065d28aa5cf3f4eef6ea0">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="f2c92a4b-fdf1-4091-a3b5-730e0262f810" xmlns:ns3="ed40aa6c-982d-4d5a-abf0-52239ff24e20" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="2f96469c0e5fa76c57eb88cc3ffabdde" ns2:_="" ns3:_="">
     <xsd:import namespace="f2c92a4b-fdf1-4091-a3b5-730e0262f810"/>
@@ -1536,10 +1548,41 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="f2c92a4b-fdf1-4091-a3b5-730e0262f810">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="ed40aa6c-982d-4d5a-abf0-52239ff24e20" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{805F7998-CA6B-4F3D-A9AA-6D44C530CD4E}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8CCAA9D4-BAE8-42AB-9344-279723EC1018}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="f2c92a4b-fdf1-4091-a3b5-730e0262f810"/>
+    <ds:schemaRef ds:uri="ed40aa6c-982d-4d5a-abf0-52239ff24e20"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -1556,20 +1599,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8CCAA9D4-BAE8-42AB-9344-279723EC1018}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{805F7998-CA6B-4F3D-A9AA-6D44C530CD4E}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="f2c92a4b-fdf1-4091-a3b5-730e0262f810"/>
-    <ds:schemaRef ds:uri="ed40aa6c-982d-4d5a-abf0-52239ff24e20"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>